<commit_message>
Add Lenin family tree data to ver3/tree.xlsx and propose new fields
- Extended person sheet with 9 new persons: maternal grandparents
  (Бланк Александр Дмитриевич, Гроссшопф Анна Ивановна), all five
  siblings (Анна, Александр, Ольга, Дмитрий, Мария Ульяновы) and
  wife Крупская Надежда Константиновна
- Added Wikidata hyperlinks for all new persons and updated existing
  entries (Илья Уляьянов Q280722, Мария Бланк Q470041)
- Added hasFather/hasMother links for Бланк Мария Александровна
  connecting her to her parents Бланк and Гроссшопф
- Extended family sheet with two new unions: Бланк+Гроссшопф and
  Ульянов_Владимир_Ильич+Крупская (married 22.07.1898, Шушенское)
- Created design/new/new_person_parameters_v1.md proposing new fields
  for person sheet (nationality_, occupation_, birthPlace_, alias_,
  wikidataId, etc.) and family sheet (endReason_, childrenCount, etc.)

Closes #74

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ver3/tree.xlsx
+++ b/ver3/tree.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32.28515625" customWidth="1" style="9" min="1" max="1"/>
@@ -647,6 +647,11 @@
           <t>1886</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>https://www.wikidata.org/wiki/Q280722</t>
+        </is>
+      </c>
     </row>
     <row r="4" customFormat="1" s="6">
       <c r="A4">
@@ -668,7 +673,16 @@
           <t>Ульянова</t>
         </is>
       </c>
-      <c r="E4" s="3" t="n"/>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Бланк_Александр_Дмитриевич</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Гроссшопф_Анна_Ивановна</t>
+        </is>
+      </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
           <t>1835</t>
@@ -691,7 +705,7 @@
       </c>
       <c r="K4" s="6" t="inlineStr">
         <is>
-          <t>https://ru.ruwiki.ru/wiki/%D0%A3%D0%BB%D1%8C%D1%8F%D0%BD%D0%BE%D0%B2%D0%B0,_%D0%9C%D0%B0%D1%80%D0%B8%D1%8F_%D0%90%D0%BB%D0%B5%D0%BA%D1%81%D0%B0%D0%BD%D0%B4%D1%80%D0%BE%D0%B2%D0%BD%D0%B0 ; https://ru.wikipedia.org/wiki/%D0%A3%D0%BB%D1%8C%D1%8F%D0%BD%D0%BE%D0%B2%D0%B0,_%D0%9C%D0%B0%D1%80%D0%B8%D1%8F_%D0%90%D0%BB%D0%B5%D0%BA%D1%81%D0%B0%D0%BD%D0%B4%D1%80%D0%BE%D0%B2%D0%BD%D0%B0</t>
+          <t>https://ru.ruwiki.ru/wiki/%D0%A3%D0%BB%D1%8C%D1%8F%D0%BD%D0%BE%D0%B2%D0%B0,_%D0%9C%D0%B0%D1%80%D0%B8%D1%8F_%D0%90%D0%BB%D0%B5%D0%BA%D1%81%D0%B0%D0%BD%D0%B4%D1%80%D0%BE%D0%B2%D0%BD%D0%B0 ; https://ru.wikipedia.org/wiki/%D0%A3%D0%BB%D1%8C%D1%8F%D0%BD%D0%BE%D0%B2%D0%B0,_%D0%9C%D0%B0%D1%80%D0%B8%D1%8F_%D0%90%D0%BB%D0%B5%D0%BA%D1%81%D0%B0%D0%BD%D0%B4%D1%80%D0%BE%D0%B2%D0%BD%D0%B0 ; https://www.wikidata.org/wiki/Q470041</t>
         </is>
       </c>
     </row>
@@ -773,17 +787,377 @@
         <f>SUBSTITUTE(B7, " ", "_")</f>
         <v/>
       </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Бланк Александр Дмитриевич</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>М</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>1804</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>1804</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>1870</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>1870</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>https://www.wikidata.org/wiki/Q29474575</t>
+        </is>
+      </c>
     </row>
     <row r="8" customFormat="1" s="6">
       <c r="A8">
         <f>SUBSTITUTE(B8, " ", "_")</f>
         <v/>
       </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Гроссшопф Анна Ивановна</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Ж</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>1799</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>1799</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>1838</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>1838</t>
+        </is>
+      </c>
     </row>
     <row r="9" customFormat="1" s="6">
       <c r="A9">
         <f>SUBSTITUTE(B9, " ", "_")</f>
         <v/>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Ульянова Анна Ильинична</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Ж</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Елизарова</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Ульянов_Илья_Николаевич</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Бланк_Мария_Александровна</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>1864</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>14.08.1864</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>1935</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>19.10.1935</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>https://www.wikidata.org/wiki/Q4174883</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <f>SUBSTITUTE(B10, " ", "_")</f>
+        <v/>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Ульянов Александр Ильич</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>М</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Ульянов_Илья_Николаевич</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Бланк_Мария_Александровна</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>1866</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>12.04.1866</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>1887</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>20.05.1887</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>https://www.wikidata.org/wiki/Q333241</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <f>SUBSTITUTE(B11, " ", "_")</f>
+        <v/>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Ульянова Ольга Ильинична</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Ж</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Ульянов_Илья_Николаевич</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Бланк_Мария_Александровна</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>1871</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>1871</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>1891</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>1891</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>https://www.wikidata.org/wiki/Q4475081</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <f>SUBSTITUTE(B12, " ", "_")</f>
+        <v/>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Ульянов Дмитрий Ильич</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>М</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Ульянов_Илья_Николаевич</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Бланк_Мария_Александровна</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>1874</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>1874</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>1943</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>1943</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>https://www.wikidata.org/wiki/Q1965609</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <f>SUBSTITUTE(B13, " ", "_")</f>
+        <v/>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Ульянова Мария Ильинична</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Ж</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Ульянов_Илья_Николаевич</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Бланк_Мария_Александровна</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>1878</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>18.02.1878</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>1937</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>12.06.1937</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>https://www.wikidata.org/wiki/Q4475079</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <f>SUBSTITUTE(B14, " ", "_")</f>
+        <v/>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Крупская Надежда Константиновна</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Ж</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>1869</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>14.02.1869</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>1939</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>27.02.1939</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>https://www.wikidata.org/wiki/Q215637</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -806,7 +1180,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="59.42578125" customWidth="1" style="9" min="1" max="1"/>
@@ -884,6 +1258,48 @@
       <c r="D2" t="inlineStr">
         <is>
           <t xml:space="preserve">25.08 (6.09) 1863 </t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <f>B3&amp;"-"&amp;C3</f>
+        <v/>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Бланк_Александр_Дмитриевич</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Гроссшопф_Анна_Ивановна</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <f>B4&amp;"-"&amp;C4</f>
+        <v/>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ульянов_Владимир_Ильич</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Крупская_Надежда_Константиновна</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>22.07.1898</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Шушенское</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add family tree data, Photo window, and new fields for issue #76
- Add siblings of Ilya Ulyanov: Vasily, Maria, Fedosya
- Add siblings of Maria Blank: Dmitry, Anna, Lyubov, Ekaterina, Sophia
- Add family record for Ульянин_Николай_Васильевич + Смирнова_Анна_Алексеевна
- Add new person fields: birthPlace_, deathPlace_, burialPlace_, occupation_
- Add new family fields: childrenCount_, endReason_
- Add Photo window (Фото) below Tree panel with folder structure
- Add translations for new fields in language sheet
- Update documentation with multiple sequential families visualization

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ver3/tree.xlsx
+++ b/ver3/tree.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:R22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32.28515625" customWidth="1" style="9" min="1" max="1"/>
@@ -545,6 +545,26 @@
           <t>patronymic</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>birthPlace_</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>deathPlace_</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>burialPlace_</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>occupation_</t>
+        </is>
+      </c>
     </row>
     <row r="2" customFormat="1" s="6">
       <c r="A2">
@@ -601,6 +621,26 @@
           <t>https://ru.wikipedia.org/wiki/%D0%9B%D0%B5%D0%BD%D0%B8%D0%BD,_%D0%92%D0%BB%D0%B0%D0%B4%D0%B8%D0%BC%D0%B8%D1%80_%D0%98%D0%BB%D1%8C%D0%B8%D1%87 ; https://www.wikidata.org/wiki/Q1394</t>
         </is>
       </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Симбирск</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Горки</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Мавзолей, Москва</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>революционер, политик</t>
+        </is>
+      </c>
     </row>
     <row r="3" customFormat="1" s="6">
       <c r="A3">
@@ -652,6 +692,21 @@
           <t>https://www.wikidata.org/wiki/Q280722</t>
         </is>
       </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Астрахань</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Симбирск</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>педагог, инспектор народных училищ</t>
+        </is>
+      </c>
     </row>
     <row r="4" customFormat="1" s="6">
       <c r="A4">
@@ -708,6 +763,21 @@
           <t>https://ru.ruwiki.ru/wiki/%D0%A3%D0%BB%D1%8C%D1%8F%D0%BD%D0%BE%D0%B2%D0%B0,_%D0%9C%D0%B0%D1%80%D0%B8%D1%8F_%D0%90%D0%BB%D0%B5%D0%BA%D1%81%D0%B0%D0%BD%D0%B4%D1%80%D0%BE%D0%B2%D0%BD%D0%B0 ; https://ru.wikipedia.org/wiki/%D0%A3%D0%BB%D1%8C%D1%8F%D0%BD%D0%BE%D0%B2%D0%B0,_%D0%9C%D0%B0%D1%80%D0%B8%D1%8F_%D0%90%D0%BB%D0%B5%D0%BA%D1%81%D0%B0%D0%BD%D0%B4%D1%80%D0%BE%D0%B2%D0%BD%D0%B0 ; https://www.wikidata.org/wiki/Q470041</t>
         </is>
       </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Санкт-Петербург</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Петроград</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>учительница</t>
+        </is>
+      </c>
     </row>
     <row r="5" customFormat="1" s="6">
       <c r="A5">
@@ -745,6 +815,21 @@
           <t>1836</t>
         </is>
       </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Нижегородская губерния</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Астрахань</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>портной, мещанин</t>
+        </is>
+      </c>
     </row>
     <row r="6" customFormat="1" s="6">
       <c r="A6">
@@ -781,6 +866,21 @@
           <t>1871</t>
         </is>
       </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Астрахань</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Астрахань</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>домохозяйка</t>
+        </is>
+      </c>
     </row>
     <row r="7" customFormat="1" s="6">
       <c r="A7">
@@ -822,6 +922,21 @@
           <t>https://www.wikidata.org/wiki/Q29474575</t>
         </is>
       </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Староконстантинов</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Кокушкино</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>врач</t>
+        </is>
+      </c>
     </row>
     <row r="8" customFormat="1" s="6">
       <c r="A8">
@@ -858,6 +973,21 @@
           <t>1838</t>
         </is>
       </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Любек, Германия</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>домохозяйка</t>
+        </is>
+      </c>
     </row>
     <row r="9" customFormat="1" s="6">
       <c r="A9">
@@ -1157,6 +1287,413 @@
       <c r="K14" t="inlineStr">
         <is>
           <t>https://www.wikidata.org/wiki/Q215637</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Ульянов Василий Николаевич</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>М</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Ульянин_Николай_Васильевич</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Смирнова_Анна_Алексеевна</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>1823</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>~1823</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>~1878</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>~1878</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>приказчик (управляющий соляным делом)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Ульянова Мария Николаевна</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Ж</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Горшкова</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Ульянин_Николай_Васильевич</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Смирнова_Анна_Алексеевна</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>~1825</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>~1825</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>домохозяйка</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Ульянова Феодосия Николаевна</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Ж</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Ульянин_Николай_Васильевич</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Смирнова_Анна_Алексеевна</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>~1827</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>~1827</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>1908</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>1908</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Бланк Дмитрий Александрович</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>М</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Бланк_Александр_Дмитриевич</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Гроссшопф_Анна_Ивановна</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>1830</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>09.09.1830</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>1850</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>19.01.1850</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Российская Империя</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Казань</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>студент юридического факультета</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Бланк Анна Александровна</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Ж</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Веретенникова</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Бланк_Александр_Дмитриевич</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Гроссшопф_Анна_Ивановна</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>1831</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>30.08.1831</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>домохозяйка</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Бланк Любовь Александровна</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Ж</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Ардашева/Пономарёва</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Бланк_Александр_Дмитриевич</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Гроссшопф_Анна_Ивановна</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>1832</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>29.08.1832</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>домохозяйка</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Бланк Екатерина Александровна</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Ж</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Залежская</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Бланк_Александр_Дмитриевич</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Гроссшопф_Анна_Ивановна</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>1834</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>04.01.1834</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>домохозяйка</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Бланк Софья Александровна</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Ж</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Лаврова</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Бланк_Александр_Дмитриевич</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Гроссшопф_Анна_Ивановна</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>1836</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>24.07.1836</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>домохозяйка</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="59.42578125" customWidth="1" style="9" min="1" max="1"/>
@@ -1239,6 +1776,16 @@
           <t>hyperLink_</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>childrenCount_</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>endReason_</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -1260,6 +1807,16 @@
           <t xml:space="preserve">25.08 (6.09) 1863 </t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>смерть супруга</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3">
@@ -1276,6 +1833,16 @@
           <t>Гроссшопф_Анна_Ивановна</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>смерть супруги</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4">
@@ -1300,6 +1867,48 @@
       <c r="E4" t="inlineStr">
         <is>
           <t>Шушенское</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>смерть супруга</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Ульянин_Николай_Васильевич</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Смирнова_Анна_Алексеевна</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>~1823</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Астрахань</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>смерть супруга</t>
         </is>
       </c>
     </row>
@@ -2322,7 +2931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7.7109375" customWidth="1" style="9" min="1" max="1"/>
@@ -3365,6 +3974,168 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>sheet</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>birthPlace_</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>место рождения</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>birthplace</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>sheet</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>deathPlace_</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>место смерти</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>place of death</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>sheet</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>burialPlace_</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>место захоронения</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>burial place</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>sheet</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>occupation_</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>профессия</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>occupation</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>sheet</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>childrenCount_</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>число детей</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>children count</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>sheet</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>endReason_</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>причина окончания</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>end reason</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="0" horizontalDpi="0" verticalDpi="0" copies="0"/>

</xml_diff>

<commit_message>
Implement v3_2data3 features for issue #78
- Add "V" button to treeview for descendants filter mode (shows spouse and descendants only)
- Add nationality_ field to person sheet in tree.xlsx
- Add marriagePlace_ field to family sheet in tree.xlsx
- Add help sheet to tree.xlsx with descriptions of all sheets and fields
- Move GraphvizOnline button to diagram bottom controls
- Add pdf and zip export buttons at diagram bottom
- Create save.js with PDF export and ZIP archive generation functions
- Color parent-child arrows: father arrows use male color, mother arrows use female color
- Increase treeview panel height by one third (45vh -> 60vh)
- Change treeview click behavior: single-click for diagram focus only, double-click opens properties
- Make diagram node selection highlight thicker (stroke-width 3 -> 5)

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ver3/tree.xlsx
+++ b/ver3/tree.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="foto_location" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="event" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="language" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="help" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="162913" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <charset val="204"/>
@@ -73,6 +74,9 @@
       <color rgb="FF000000"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -95,7 +99,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -112,6 +116,10 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -456,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R22"/>
+  <dimension ref="A1:S22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32.28515625" customWidth="1" style="9" min="1" max="1"/>
@@ -565,6 +573,11 @@
           <t>occupation_</t>
         </is>
       </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>nationality_</t>
+        </is>
+      </c>
     </row>
     <row r="2" customFormat="1" s="6">
       <c r="A2">
@@ -1430,7 +1443,6 @@
           <t>1908</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="B18" t="inlineStr">
@@ -1717,7 +1729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="59.42578125" customWidth="1" style="9" min="1" max="1"/>
@@ -1784,6 +1796,11 @@
       <c r="K1" t="inlineStr">
         <is>
           <t>endReason_</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>marriagePlace_</t>
         </is>
       </c>
     </row>
@@ -2931,7 +2948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7.7109375" customWidth="1" style="9" min="1" max="1"/>
@@ -4136,8 +4153,1860 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>nationality_</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Национальность</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Nationality</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>marriagePlace_</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Место брака</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Marriage place</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="0" horizontalDpi="0" verticalDpi="0" copies="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C107"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" style="9" min="1" max="1"/>
+    <col width="20" customWidth="1" style="9" min="2" max="2"/>
+    <col width="60" customWidth="1" style="9" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>Лист (Sheet)</t>
+        </is>
+      </c>
+      <c r="B1" s="12" t="inlineStr">
+        <is>
+          <t>Поле (Field)</t>
+        </is>
+      </c>
+      <c r="C1" s="12" t="inlineStr">
+        <is>
+          <t>Описание (Description)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
+      <c r="C2" s="13" t="inlineStr">
+        <is>
+          <t>Лист персон (людей) семейного древа</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>idA</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>Уникальный идентификатор персоны (без пробелов)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>label_</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>Полное имя персоны (ФИО)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>sex</t>
+        </is>
+      </c>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>Пол: М (мужской) или Ж (женский)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>surName2_</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>Девичья фамилия (для женщин, вышедших замуж)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>hasFather</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>idA отца персоны</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>hasMother</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>idA матери персоны</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>birth</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>Год рождения</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>birthFull_</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>Полная дата рождения</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>death</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>Год смерти</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>deathFull_</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>Полная дата смерти</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>hyperLink_</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>Ссылки на внешние источники (через ;)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>surName</t>
+        </is>
+      </c>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>Фамилия</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>firstName</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>Имя</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>patronymic</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>Отчество</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>birthPlace_</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>Место рождения</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>deathPlace_</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>Место смерти</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>burialPlace_</t>
+        </is>
+      </c>
+      <c r="C19" s="13" t="inlineStr">
+        <is>
+          <t>Место захоронения</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>occupation_</t>
+        </is>
+      </c>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>Род занятий, профессия</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>person</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>nationality_</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>Национальность</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="C22" s="13" t="inlineStr">
+        <is>
+          <t>Лист семей (браков)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>idA</t>
+        </is>
+      </c>
+      <c r="C23" s="13" t="inlineStr">
+        <is>
+          <t>Уникальный идентификатор семьи</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>husband</t>
+        </is>
+      </c>
+      <c r="C24" s="13" t="inlineStr">
+        <is>
+          <t>idA мужа</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>wife</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>idA жены</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>marriage_</t>
+        </is>
+      </c>
+      <c r="C26" s="13" t="inlineStr">
+        <is>
+          <t>Год заключения брака</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>marriagePlace_</t>
+        </is>
+      </c>
+      <c r="C27" s="13" t="inlineStr">
+        <is>
+          <t>Место заключения брака</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>locationM_</t>
+        </is>
+      </c>
+      <c r="C28" s="13" t="inlineStr">
+        <is>
+          <t>Основные места жизни семьи (через ;)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>divorce</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>Год развода</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>locationD</t>
+        </is>
+      </c>
+      <c r="C30" s="13" t="inlineStr">
+        <is>
+          <t>Место развода</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>label_</t>
+        </is>
+      </c>
+      <c r="C31" s="13" t="inlineStr">
+        <is>
+          <t>Подпись семьи на диаграмме</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>hyperLink_</t>
+        </is>
+      </c>
+      <c r="C32" s="13" t="inlineStr">
+        <is>
+          <t>Ссылки на внешние источники (через ;)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>childrenCount_</t>
+        </is>
+      </c>
+      <c r="C33" s="13" t="inlineStr">
+        <is>
+          <t>Количество детей</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>family</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>endReason_</t>
+        </is>
+      </c>
+      <c r="C34" s="13" t="inlineStr">
+        <is>
+          <t>Причина окончания брака</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>foto_person</t>
+        </is>
+      </c>
+      <c r="C35" s="13" t="inlineStr">
+        <is>
+          <t>Лист фотографий персон</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>foto_person</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>id_person</t>
+        </is>
+      </c>
+      <c r="C36" s="13" t="inlineStr">
+        <is>
+          <t>idA персоны</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>foto_person</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>suffix</t>
+        </is>
+      </c>
+      <c r="C37" s="13" t="inlineStr">
+        <is>
+          <t>Суффикс файла (год фото)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>foto_person</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="C38" s="13" t="inlineStr">
+        <is>
+          <t>Расширение файла (jpg, png)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>foto_person</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>idA</t>
+        </is>
+      </c>
+      <c r="C39" s="13" t="inlineStr">
+        <is>
+          <t>Имя файла фото (вычисляется автоматически)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>foto_person</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>title_</t>
+        </is>
+      </c>
+      <c r="C40" s="13" t="inlineStr">
+        <is>
+          <t>Название/описание фото</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>foto_person</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>location_</t>
+        </is>
+      </c>
+      <c r="C41" s="13" t="inlineStr">
+        <is>
+          <t>Место съёмки</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>foto_person</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>date_</t>
+        </is>
+      </c>
+      <c r="C42" s="13" t="inlineStr">
+        <is>
+          <t>Дата съёмки</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>foto_person</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>label_</t>
+        </is>
+      </c>
+      <c r="C43" s="13" t="inlineStr">
+        <is>
+          <t>Подпись к фото</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>foto_person</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>hyperLink_</t>
+        </is>
+      </c>
+      <c r="C44" s="13" t="inlineStr">
+        <is>
+          <t>Ссылка на источник фото</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>foto_family</t>
+        </is>
+      </c>
+      <c r="C45" s="13" t="inlineStr">
+        <is>
+          <t>Лист семейных фотографий</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>foto_family</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>id_family</t>
+        </is>
+      </c>
+      <c r="C46" s="13" t="inlineStr">
+        <is>
+          <t>idA семьи</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>foto_family</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>suffix_</t>
+        </is>
+      </c>
+      <c r="C47" s="13" t="inlineStr">
+        <is>
+          <t>Суффикс файла (год фото)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>foto_family</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="C48" s="13" t="inlineStr">
+        <is>
+          <t>Расширение файла</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>foto_family</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>idA</t>
+        </is>
+      </c>
+      <c r="C49" s="13" t="inlineStr">
+        <is>
+          <t>Имя файла фото</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>foto_family</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>title_</t>
+        </is>
+      </c>
+      <c r="C50" s="13" t="inlineStr">
+        <is>
+          <t>Название фото</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>foto_family</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>inFamily</t>
+        </is>
+      </c>
+      <c r="C51" s="13" t="inlineStr">
+        <is>
+          <t>Кто из семьи на фото</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>foto_family</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>inFoto</t>
+        </is>
+      </c>
+      <c r="C52" s="13" t="inlineStr">
+        <is>
+          <t>Кто изображён на фото</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>foto_family</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>full_person</t>
+        </is>
+      </c>
+      <c r="C53" s="13" t="inlineStr">
+        <is>
+          <t>Полный список персон</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>foto_family</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>location_</t>
+        </is>
+      </c>
+      <c r="C54" s="13" t="inlineStr">
+        <is>
+          <t>Место съёмки</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>foto_family</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>date_</t>
+        </is>
+      </c>
+      <c r="C55" s="13" t="inlineStr">
+        <is>
+          <t>Дата съёмки</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>foto_family</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>person_label</t>
+        </is>
+      </c>
+      <c r="C56" s="13" t="inlineStr">
+        <is>
+          <t>Подписи персон</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>foto_family</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>label_</t>
+        </is>
+      </c>
+      <c r="C57" s="13" t="inlineStr">
+        <is>
+          <t>Подпись к фото</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>foto_family</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>hyperLink_</t>
+        </is>
+      </c>
+      <c r="C58" s="13" t="inlineStr">
+        <is>
+          <t>Ссылка на источник</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>foto_family</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>id_personAll</t>
+        </is>
+      </c>
+      <c r="C59" s="13" t="inlineStr">
+        <is>
+          <t>Все idA персон на фото (через ;)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>foto_group</t>
+        </is>
+      </c>
+      <c r="C60" s="13" t="inlineStr">
+        <is>
+          <t>Лист групповых фотографий</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>foto_group</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>id_person</t>
+        </is>
+      </c>
+      <c r="C61" s="13" t="inlineStr">
+        <is>
+          <t>idA основной персоны</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>foto_group</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>suffix_</t>
+        </is>
+      </c>
+      <c r="C62" s="13" t="inlineStr">
+        <is>
+          <t>Суффикс файла</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>foto_group</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="C63" s="13" t="inlineStr">
+        <is>
+          <t>Расширение файла</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>foto_group</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>idA</t>
+        </is>
+      </c>
+      <c r="C64" s="13" t="inlineStr">
+        <is>
+          <t>Имя файла фото</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>foto_group</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>title_</t>
+        </is>
+      </c>
+      <c r="C65" s="13" t="inlineStr">
+        <is>
+          <t>Название фото</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>foto_group</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>id_personAll</t>
+        </is>
+      </c>
+      <c r="C66" s="13" t="inlineStr">
+        <is>
+          <t>Все idA персон на фото (через ;)</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>foto_group</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>location_</t>
+        </is>
+      </c>
+      <c r="C67" s="13" t="inlineStr">
+        <is>
+          <t>Место съёмки</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>foto_group</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>date_</t>
+        </is>
+      </c>
+      <c r="C68" s="13" t="inlineStr">
+        <is>
+          <t>Дата съёмки</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>foto_group</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>person_label</t>
+        </is>
+      </c>
+      <c r="C69" s="13" t="inlineStr">
+        <is>
+          <t>Подписи персон</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>foto_group</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>label_</t>
+        </is>
+      </c>
+      <c r="C70" s="13" t="inlineStr">
+        <is>
+          <t>Подпись к фото</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>foto_group</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>hyperLink_</t>
+        </is>
+      </c>
+      <c r="C71" s="13" t="inlineStr">
+        <is>
+          <t>Ссылка на источник</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>foto_location</t>
+        </is>
+      </c>
+      <c r="C72" s="13" t="inlineStr">
+        <is>
+          <t>Лист фотографий мест</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>foto_location</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>id_loc</t>
+        </is>
+      </c>
+      <c r="C73" s="13" t="inlineStr">
+        <is>
+          <t>Идентификатор места</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>foto_location</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>suffix</t>
+        </is>
+      </c>
+      <c r="C74" s="13" t="inlineStr">
+        <is>
+          <t>Суффикс файла</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>foto_location</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>extension</t>
+        </is>
+      </c>
+      <c r="C75" s="13" t="inlineStr">
+        <is>
+          <t>Расширение файла</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>foto_location</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>idA</t>
+        </is>
+      </c>
+      <c r="C76" s="13" t="inlineStr">
+        <is>
+          <t>Имя файла фото</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>foto_location</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>title_</t>
+        </is>
+      </c>
+      <c r="C77" s="13" t="inlineStr">
+        <is>
+          <t>Название места</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>foto_location</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>locationGroup</t>
+        </is>
+      </c>
+      <c r="C78" s="13" t="inlineStr">
+        <is>
+          <t>Группа мест</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>foto_location</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>id_personAll</t>
+        </is>
+      </c>
+      <c r="C79" s="13" t="inlineStr">
+        <is>
+          <t>Связанные персоны (через ;)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>foto_location</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>id_familyAll</t>
+        </is>
+      </c>
+      <c r="C80" s="13" t="inlineStr">
+        <is>
+          <t>Связанные семьи (через ;)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>foto_location</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>location_</t>
+        </is>
+      </c>
+      <c r="C81" s="13" t="inlineStr">
+        <is>
+          <t>Адрес/описание места</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>foto_location</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>date_</t>
+        </is>
+      </c>
+      <c r="C82" s="13" t="inlineStr">
+        <is>
+          <t>Дата съёмки</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>foto_location</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>person_label</t>
+        </is>
+      </c>
+      <c r="C83" s="13" t="inlineStr">
+        <is>
+          <t>Подписи персон</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>foto_location</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>label_</t>
+        </is>
+      </c>
+      <c r="C84" s="13" t="inlineStr">
+        <is>
+          <t>Подпись к фото</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>foto_location</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>hyperLink_</t>
+        </is>
+      </c>
+      <c r="C85" s="13" t="inlineStr">
+        <is>
+          <t>Ссылка на источник</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>foto_location</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>synonym_</t>
+        </is>
+      </c>
+      <c r="C86" s="13" t="inlineStr">
+        <is>
+          <t>Синонимы названия места</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>event</t>
+        </is>
+      </c>
+      <c r="C87" s="13" t="inlineStr">
+        <is>
+          <t>Лист событий</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>event</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>id_event</t>
+        </is>
+      </c>
+      <c r="C88" s="13" t="inlineStr">
+        <is>
+          <t>Идентификатор события</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>event</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>eventGroup</t>
+        </is>
+      </c>
+      <c r="C89" s="13" t="inlineStr">
+        <is>
+          <t>Группа/тип события</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>event</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>id_personAll</t>
+        </is>
+      </c>
+      <c r="C90" s="13" t="inlineStr">
+        <is>
+          <t>Участники события (через ;)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>event</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>id_familyAll</t>
+        </is>
+      </c>
+      <c r="C91" s="13" t="inlineStr">
+        <is>
+          <t>Связанные семьи (через ;)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>event</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>title_</t>
+        </is>
+      </c>
+      <c r="C92" s="13" t="inlineStr">
+        <is>
+          <t>Название события</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>event</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>location_</t>
+        </is>
+      </c>
+      <c r="C93" s="13" t="inlineStr">
+        <is>
+          <t>Место события</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>event</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>date_</t>
+        </is>
+      </c>
+      <c r="C94" s="13" t="inlineStr">
+        <is>
+          <t>Дата события</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>event</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>person_label</t>
+        </is>
+      </c>
+      <c r="C95" s="13" t="inlineStr">
+        <is>
+          <t>Подписи участников</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>event</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>label_</t>
+        </is>
+      </c>
+      <c r="C96" s="13" t="inlineStr">
+        <is>
+          <t>Описание события</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>event</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>hyperLink_</t>
+        </is>
+      </c>
+      <c r="C97" s="13" t="inlineStr">
+        <is>
+          <t>Ссылки на источники</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>event</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>foto_person</t>
+        </is>
+      </c>
+      <c r="C98" s="13" t="inlineStr">
+        <is>
+          <t>Файл фото персоны</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>event</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>foto_family</t>
+        </is>
+      </c>
+      <c r="C99" s="13" t="inlineStr">
+        <is>
+          <t>Файл семейного фото</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>event</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>foto_group</t>
+        </is>
+      </c>
+      <c r="C100" s="13" t="inlineStr">
+        <is>
+          <t>Файл группового фото</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>event</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>foto_location</t>
+        </is>
+      </c>
+      <c r="C101" s="13" t="inlineStr">
+        <is>
+          <t>Файл фото места</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>language</t>
+        </is>
+      </c>
+      <c r="C102" s="13" t="inlineStr">
+        <is>
+          <t>Лист локализации (переводов полей)</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>language</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
+      <c r="C103" s="13" t="inlineStr">
+        <is>
+          <t>Тип записи</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>language</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>object</t>
+        </is>
+      </c>
+      <c r="C104" s="13" t="inlineStr">
+        <is>
+          <t>Название листа</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>language</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C105" s="13" t="inlineStr">
+        <is>
+          <t>Название поля (с суффиксом _)</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>language</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>ru</t>
+        </is>
+      </c>
+      <c r="C106" s="13" t="inlineStr">
+        <is>
+          <t>Перевод на русский</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>language</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C107" s="13" t="inlineStr">
+        <is>
+          <t>Перевод на английский</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>